<commit_message>
chore(kl2): redact Rotan-1 exact depths and TWT from outputs (AMANAH)
Removes exact pick depths (NN12/NN11/NN10, Landmark tops), top reservoir
and GWC depths, TWT@TD, VSP parameters and the MD->TVDSS factor from the
v3 penetration scaffold; regenerates the v3 xlsx and chart. Rotan-1
seabed/TD kept as public values (Oil & Gas Journal, 5 Feb 2007).

Adds a provenance README (v2 row = known fixture fault; wells_summary.json
and qc_samples.csv are DER_SYNTHETIC fixtures) and a deny-by-default
.gitignore for this folder. Git history intentionally not rewritten
(ARIF decision 2026-10-15).

REPO=geox
</commit_message>
<xml_diff>
--- a/outputs/kl2_kinabalu/kl2_kinabalu_well_data_v3.xlsx
+++ b/outputs/kl2_kinabalu/kl2_kinabalu_well_data_v3.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wells" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NN_Horizon_Picks" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datum" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provenance" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Wells" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="NN_Horizon_Picks" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Datum" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Provenance" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -591,13 +591,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2114.7</v>
-      </c>
-      <c r="E4" t="n">
-        <v>2660</v>
-      </c>
+        <v>2141</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1149.4</v>
+        <v>1150</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -611,7 +609,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>REAL [RELAY-ENT WCR/Geoservice]</t>
+          <t>PUBLIC [OGJ 2007]</t>
         </is>
       </c>
       <c r="J4" t="n">
@@ -2394,7 +2392,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>REAL-BIO</t>
+          <t>REAL-BIO (depth REDACTED)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
@@ -2434,31 +2432,19 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>REAL-BIO</t>
-        </is>
-      </c>
-      <c r="G34" t="n">
-        <v>1969.4</v>
-      </c>
-      <c r="H34" t="n">
-        <v>48</v>
-      </c>
-      <c r="I34" t="n">
-        <v>248.5</v>
-      </c>
-      <c r="J34" t="n">
-        <v>253.1</v>
-      </c>
+          <t>REAL-BIO (depth REDACTED)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="L34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2486,21 +2472,13 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>REAL-BIO</t>
-        </is>
-      </c>
-      <c r="G35" t="n">
-        <v>1813.8</v>
-      </c>
-      <c r="H35" t="n">
-        <v>32.1</v>
-      </c>
-      <c r="I35" t="n">
-        <v>240.7</v>
-      </c>
-      <c r="J35" t="n">
-        <v>242.8</v>
-      </c>
+          <t>REAL-BIO (depth REDACTED)</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2538,16 +2516,16 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>1555.4</v>
+        <v>1566.8</v>
       </c>
       <c r="H36" t="n">
         <v>68.3</v>
       </c>
       <c r="I36" t="n">
-        <v>333.3</v>
+        <v>334.3</v>
       </c>
       <c r="J36" t="n">
-        <v>340.2</v>
+        <v>341.2</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
@@ -2586,16 +2564,16 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>1530</v>
+        <v>1540.8</v>
       </c>
       <c r="H37" t="n">
         <v>65.3</v>
       </c>
       <c r="I37" t="n">
-        <v>331.1</v>
+        <v>332.1</v>
       </c>
       <c r="J37" t="n">
-        <v>337.5</v>
+        <v>338.4</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -2634,16 +2612,16 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>1525</v>
+        <v>1535.6</v>
       </c>
       <c r="H38" t="n">
         <v>64.7</v>
       </c>
       <c r="I38" t="n">
-        <v>330.7</v>
+        <v>331.6</v>
       </c>
       <c r="J38" t="n">
-        <v>337</v>
+        <v>337.9</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
@@ -2682,16 +2660,16 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>1392</v>
+        <v>1399.1</v>
       </c>
       <c r="H39" t="n">
         <v>48.9</v>
       </c>
       <c r="I39" t="n">
-        <v>319.3</v>
+        <v>319.9</v>
       </c>
       <c r="J39" t="n">
-        <v>323</v>
+        <v>323.6</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
@@ -2730,16 +2708,16 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>1175.8</v>
+        <v>1177.1</v>
       </c>
       <c r="H40" t="n">
         <v>23.1</v>
       </c>
       <c r="I40" t="n">
-        <v>300.8</v>
+        <v>300.9</v>
       </c>
       <c r="J40" t="n">
-        <v>301.7</v>
+        <v>301.8</v>
       </c>
       <c r="K40" t="inlineStr">
         <is>
@@ -6198,34 +6176,34 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Rotan-1 header (seabed/TD/TWT)</t>
+          <t>Rotan-1 header (seabed/TD)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>REAL [RELAY-ENT]</t>
+          <t>PUBLIC</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>WCR Rotan-1 via KL2_Wells_Data_Compilation.xlsx WELL_HEADERS/FORMATION_TOPS (Geoservice); VSP tie 0.85</t>
+          <t>Oil &amp; Gas Journal, 5 Feb 2007 (Murphy Oil): TD 7,024 ft in 3,773 ft of water; TWT@TD REDACTED</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Rotan-1 NN picks</t>
+          <t>Rotan-1 NN picks / tops / pay / GWC</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>REAL [RELAY-ENT]</t>
+          <t>REAL [RELAY-ENT] — depths REDACTED 2026-10-15</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>KL2_SOURCE_OF_TRUTH_MASTER.xlsx BIO_ZONE_INTERVALS + KL2V2 Landmark; MD-&gt;TVDSS x0.98772 [DER]</t>
+          <t>enterprise relay (WCR + biostrat + Landmark); exact values held outside repo</t>
         </is>
       </c>
     </row>
@@ -6305,12 +6283,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DER — 200-500 m (Rotan REAL: 150 m + 0.05z, VSP-constrained)</t>
+          <t>DER — 200-500 m</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>NSPW mobile-shale province; VSI VSP 106 shots for Rotan</t>
+          <t>NSPW mobile-shale province; Rotan VSP details REDACTED</t>
         </is>
       </c>
     </row>

</xml_diff>